<commit_message>
Remove PowerPoint generation and integrate CLIP multimodal meme analysis into Streamlit dashboard
</commit_message>
<xml_diff>
--- a/Milan Loi - Suivi de stage BUT2.xlsx
+++ b/Milan Loi - Suivi de stage BUT2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/milan/projects/rgu-internship-social-media-analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FCC84D6-864F-A740-B079-A43840726C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0FC0805-AED5-DC48-B6F1-56926543151C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="200" yWindow="840" windowWidth="29000" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t>Nom :</t>
   </si>
@@ -116,6 +116,54 @@
   </si>
   <si>
     <t>Rappel du sujet : we vs them social media analysis</t>
+  </si>
+  <si>
+    <t>Intégration de la Perspective API de Google pour le scoring de toxicité. Calcul de l'Indice de Polarisation par communauté. Génération de cartes de chaleur (heatmaps) de distribution.</t>
+  </si>
+  <si>
+    <t>Conception du squelette de l'application Streamlit. Intégration des filtres de données (plateformes, dates, thématiques) dans la barre latérale. Développement de l'onglet de comparaison inter-plateformes.</t>
+  </si>
+  <si>
+    <t>Intégration des graphiques Plotly/Altair (séries temporelles et distribution de la toxicité). Tests d'assurance qualité (QA) de l'application Streamlit (cas limites, réactivité des filtres). Présentation devant le groupe de recherche</t>
+  </si>
+  <si>
+    <t>Rédaction du rapport. Documentation complète du code source (docstrings, typage strict et fichier README.md). Modélisation des flux de données du tableau de bord (diagramme d'architecture).</t>
+  </si>
+  <si>
+    <t>Finaliser la version 1.0 du tableau de bord interactif pour sa livraison aux chercheurs non-informaticiens du groupe et le présenter au groupe</t>
+  </si>
+  <si>
+    <t>Mettre en place l'infrastructure front-end du tableau de bord pour permettre une exploration interactive des données.</t>
+  </si>
+  <si>
+    <t>Quantifier la toxicité contextuelle et lier la prévalence du discours "Nous vs Eux" (pronoms exclusifs) à la polarisation.</t>
+  </si>
+  <si>
+    <t>Latence et quotas de requêtes lors de l'appel à l'API externe sur l'ensemble du dataset.</t>
+  </si>
+  <si>
+    <t>Implémentation d'un système de requêtes asynchrones par lots (batching) et mise en cache des scores de toxicité.</t>
+  </si>
+  <si>
+    <t>Surcharge de l'interface graphique lors de l'affichage de visualisations de réseaux trop denses.</t>
+  </si>
+  <si>
+    <t>Utilisation de techniques de filtrage en amont (par niveau de modularité minimum) pour alléger le rendu du graphe.</t>
+  </si>
+  <si>
+    <t>Débogage des flux de données réactifs (states) de Streamlit lors de changements rapides de filtres imbriqués.</t>
+  </si>
+  <si>
+    <t>Utilisation du décorateur @st.cache_data pour figer les calculs lourds et structuration d'un journal d'anomalies.</t>
+  </si>
+  <si>
+    <t>Difficulté à synthétiser et formaliser rigoureusement les concepts mathématiques (Louvain, modularité) en français.</t>
+  </si>
+  <si>
+    <t>Simplification des concepts afin d'être compris</t>
+  </si>
+  <si>
+    <t>Produire les livrables académiques écrits et stabiliser la documentation technique pour la reproductibilité du projet.</t>
   </si>
 </sst>
 </file>
@@ -222,14 +270,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -504,11 +552,11 @@
       </c>
     </row>
     <row r="3" spans="1:6" s="1" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
     </row>
     <row r="4" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
@@ -609,49 +657,81 @@
       <c r="C9" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="12" t="s">
         <v>28</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>6</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="4"/>
+      <c r="B10" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>40</v>
+      </c>
       <c r="F10" s="7"/>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>7</v>
       </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B11" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="64" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>8</v>
       </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B12" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>9</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
+      <c r="B13" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="3">

</xml_diff>